<commit_message>
[doc] (journal de travail) Update journal de travail
</commit_message>
<xml_diff>
--- a/WIP/journaux de travaux/CI_CD_journalTravail_Belkhiria_Sofiene_Test.xlsx
+++ b/WIP/journaux de travaux/CI_CD_journalTravail_Belkhiria_Sofiene_Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\po66qga\Documents\GitHub\P_DevOps324-450\WIP\journaux de travaux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CAA9BAA-B35F-4208-9EC7-A1313CB6CE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EF85F7-2D93-4145-96E1-8E009B4B9D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="50">
   <si>
     <t>Auteur:</t>
   </si>
@@ -188,6 +188,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ecriture de la partie test backend du rapport </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finalisation de la partie test unitaire du backend </t>
   </si>
 </sst>
 </file>
@@ -1146,7 +1149,7 @@
                   <c:v>525</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>335</c:v>
+                  <c:v>495</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1989,16 +1992,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>2.2727272727272728E-2</c:v>
+                  <c:v>1.9230769230769232E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.59659090909090906</c:v>
+                  <c:v>0.50480769230769229</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.38068181818181818</c:v>
+                  <c:v>0.47596153846153844</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4233,7 +4236,7 @@
       <c r="B3" s="83"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>17 heures 40 minutes</v>
+        <v>20 heures 20 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4248,15 +4251,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>600</v>
+        <v>720</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>460</v>
+        <v>500</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>1060</v>
+        <v>1220</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4733,15 +4736,25 @@
       <c r="G24" s="45"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="74" t="str">
+      <c r="A25" s="74">
         <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="40"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="28"/>
+        <v>2</v>
+      </c>
+      <c r="B25" s="40">
+        <v>45663</v>
+      </c>
+      <c r="C25" s="41">
+        <v>2</v>
+      </c>
+      <c r="D25" s="42">
+        <v>40</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>49</v>
+      </c>
       <c r="G25" s="46"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -10979,7 +10992,7 @@
       </c>
       <c r="G6" s="47">
         <f>SUM(A6:B6)/$C$10</f>
-        <v>2.2727272727272728E-2</v>
+        <v>1.9230769230769232E-2</v>
       </c>
       <c r="L6" s="62" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11053,7 +11066,7 @@
       </c>
       <c r="G8" s="47">
         <f t="shared" si="2"/>
-        <v>0.59659090909090906</v>
+        <v>0.50480769230769229</v>
       </c>
       <c r="L8" s="65" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11070,15 +11083,15 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>215</v>
+        <v>255</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>335</v>
+        <v>495</v>
       </c>
       <c r="E9" s="23" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11086,11 +11099,11 @@
       </c>
       <c r="F9" s="55" t="str">
         <f t="shared" si="1"/>
-        <v>5 h 35 min</v>
+        <v>8 h 15 min</v>
       </c>
       <c r="G9" s="56">
         <f t="shared" si="2"/>
-        <v>0.38068181818181818</v>
+        <v>0.47596153846153844</v>
       </c>
       <c r="L9" s="66" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11107,26 +11120,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>420</v>
+        <v>540</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>460</v>
+        <v>500</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>880</v>
+        <v>1040</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>14 h 40 min</v>
+        <v>17 h 20 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.16666666666666666</v>
+        <v>0.19696969696969696</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11165,12 +11178,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11397,20 +11412,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11435,18 +11457,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>